<commit_message>
[removed] sample run logs
</commit_message>
<xml_diff>
--- a/Testkit_Q1_PRN222/Q11/TC1/Detail.xlsx
+++ b/Testkit_Q1_PRN222/Q11/TC1/Detail.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\School\SEP490\networking\QuestionQ1_FA25\Testkit_Q1_PRN222\Q11\TC1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\School\NET\auto-grading\Testkit_Q1_PRN222\Q11\TC1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BEA96F2-7592-404E-8E8D-F0A1B7C2E352}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB4A90C-BE3E-4D57-9556-5DBD21D88E22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User" sheetId="1" r:id="rId1"/>
@@ -44,9 +44,6 @@
     <t>StartServer</t>
   </si>
   <si>
-    <t xml:space="preserve"> 5 + 4</t>
-  </si>
-  <si>
     <t>Time</t>
   </si>
   <si>
@@ -102,6 +99,9 @@
   </si>
   <si>
     <t>Server responding (SYN-ACK)</t>
+  </si>
+  <si>
+    <t>5 + 4</t>
   </si>
 </sst>
 </file>
@@ -528,7 +528,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>1</v>
@@ -579,31 +579,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
@@ -611,29 +611,29 @@
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>21</v>
       </c>
       <c r="H2" s="3"/>
       <c r="I2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -641,29 +641,29 @@
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="F3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>25</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>